<commit_message>
Fix meeting dates and add overall plan
</commit_message>
<xml_diff>
--- a/Шаблон плана МОП.xlsx
+++ b/Шаблон плана МОП.xlsx
@@ -27,7 +27,7 @@
       <name val="Calibri"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -43,6 +43,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFEAF3FF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFEDE7FF"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -74,7 +80,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0"/>
@@ -86,6 +92,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
 </styleSheet>
@@ -93,7 +102,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F13"/>
+  <dimension ref="A1:F14"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="28" customWidth="1"/>
@@ -147,22 +156,22 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="22" customHeight="1">
-      <c r="A4" t="inlineStr" s="4">
-        <is>
-          <t>Черткова Ирина</t>
-        </is>
-      </c>
-      <c r="B4" s="5"/>
-      <c r="C4" s="5"/>
-      <c r="D4" s="5"/>
-      <c r="E4" s="5"/>
-      <c r="F4" s="5"/>
+    <row r="4" ht="24" customHeight="1">
+      <c r="A4" t="inlineStr" s="6">
+        <is>
+          <t>Общий план</t>
+        </is>
+      </c>
+      <c r="B4" s="6"/>
+      <c r="C4" s="6"/>
+      <c r="D4" s="6"/>
+      <c r="E4" s="6"/>
+      <c r="F4" s="6"/>
     </row>
     <row r="5" ht="22" customHeight="1">
       <c r="A5" t="inlineStr" s="4">
         <is>
-          <t>Газисова Мария</t>
+          <t>Черткова Ирина</t>
         </is>
       </c>
       <c r="B5" s="5"/>
@@ -174,7 +183,7 @@
     <row r="6" ht="22" customHeight="1">
       <c r="A6" t="inlineStr" s="4">
         <is>
-          <t>Попова Олеся</t>
+          <t>Газисова Мария</t>
         </is>
       </c>
       <c r="B6" s="5"/>
@@ -186,7 +195,7 @@
     <row r="7" ht="22" customHeight="1">
       <c r="A7" t="inlineStr" s="4">
         <is>
-          <t>Попова Юлия</t>
+          <t>Попова Олеся</t>
         </is>
       </c>
       <c r="B7" s="5"/>
@@ -198,7 +207,7 @@
     <row r="8" ht="22" customHeight="1">
       <c r="A8" t="inlineStr" s="4">
         <is>
-          <t>Губайдулина Заррина</t>
+          <t>Попова Юлия</t>
         </is>
       </c>
       <c r="B8" s="5"/>
@@ -210,7 +219,7 @@
     <row r="9" ht="22" customHeight="1">
       <c r="A9" t="inlineStr" s="4">
         <is>
-          <t>Тончу Ростислав</t>
+          <t>Губайдулина Заррина</t>
         </is>
       </c>
       <c r="B9" s="5"/>
@@ -222,7 +231,7 @@
     <row r="10" ht="22" customHeight="1">
       <c r="A10" t="inlineStr" s="4">
         <is>
-          <t>Погребинский Артем</t>
+          <t>Тончу Ростислав</t>
         </is>
       </c>
       <c r="B10" s="5"/>
@@ -234,7 +243,7 @@
     <row r="11" ht="22" customHeight="1">
       <c r="A11" t="inlineStr" s="4">
         <is>
-          <t>Камболин Александр</t>
+          <t>Погребинский Артем</t>
         </is>
       </c>
       <c r="B11" s="5"/>
@@ -246,7 +255,7 @@
     <row r="12" ht="22" customHeight="1">
       <c r="A12" t="inlineStr" s="4">
         <is>
-          <t>Жуков Лев</t>
+          <t>Камболин Александр</t>
         </is>
       </c>
       <c r="B12" s="5"/>
@@ -258,7 +267,7 @@
     <row r="13" ht="22" customHeight="1">
       <c r="A13" t="inlineStr" s="4">
         <is>
-          <t>Гавриленко Елена</t>
+          <t>Жуков Лев</t>
         </is>
       </c>
       <c r="B13" s="5"/>
@@ -267,7 +276,19 @@
       <c r="E13" s="5"/>
       <c r="F13" s="5"/>
     </row>
+    <row r="14" ht="22" customHeight="1">
+      <c r="A14" t="inlineStr" s="4">
+        <is>
+          <t>Гавриленко Елена</t>
+        </is>
+      </c>
+      <c r="B14" s="5"/>
+      <c r="C14" s="5"/>
+      <c r="D14" s="5"/>
+      <c r="E14" s="5"/>
+      <c r="F14" s="5"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A3:F13"/>
+  <autoFilter ref="A3:F14"/>
 </worksheet>
 </file>
</xml_diff>